<commit_message>
Add complete sample dataset with 20 assets
</commit_message>
<xml_diff>
--- a/IT Asset Inventory.xlsx
+++ b/IT Asset Inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bilal Akhtar\Documents\it-asset-inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BFE892-402B-40E0-9366-067C81AE400C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAF4A01-9F07-4564-82A8-B3B9D0C4C30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="142">
   <si>
     <t>Asset Tag</t>
   </si>
@@ -78,6 +78,321 @@
     <t>In Use</t>
   </si>
   <si>
+    <t>7K2L9X3</t>
+  </si>
+  <si>
+    <t>5CD2371XYZ</t>
+  </si>
+  <si>
+    <t>PF3K9RT2</t>
+  </si>
+  <si>
+    <t>9M4P2WQ1</t>
+  </si>
+  <si>
+    <t>HP EliteBook 840 G9</t>
+  </si>
+  <si>
+    <t>Lenovo ThinkPad T14</t>
+  </si>
+  <si>
+    <t>Dell Latitude 7420</t>
+  </si>
+  <si>
+    <t>James Johnson</t>
+  </si>
+  <si>
+    <t>John Williams</t>
+  </si>
+  <si>
+    <t>Robert Brown</t>
+  </si>
+  <si>
+    <t>David Jones</t>
+  </si>
+  <si>
+    <t>William Garcia</t>
+  </si>
+  <si>
+    <t>Mary Miller</t>
+  </si>
+  <si>
+    <t>Maria Davis</t>
+  </si>
+  <si>
+    <t>Joseph Martinez</t>
+  </si>
+  <si>
+    <t>Bilal Akhtar</t>
+  </si>
+  <si>
+    <t>Maya Bennett</t>
+  </si>
+  <si>
+    <t>Ava Collins</t>
+  </si>
+  <si>
+    <t>Layla Cooper</t>
+  </si>
+  <si>
+    <t>Owen Blake</t>
+  </si>
+  <si>
+    <t>Jane Doe</t>
+  </si>
+  <si>
+    <t>Noah Parker</t>
+  </si>
+  <si>
+    <t>Ethan Brooks</t>
+  </si>
+  <si>
+    <t>Mason Wright</t>
+  </si>
+  <si>
+    <t>Aria Sullivan</t>
+  </si>
+  <si>
+    <t>Chloe Reed</t>
+  </si>
+  <si>
+    <t>bilal.akhtar@itproject.ca</t>
+  </si>
+  <si>
+    <t>james.johnson@itproject.ca</t>
+  </si>
+  <si>
+    <t>john.williams@itproject.ca</t>
+  </si>
+  <si>
+    <t>robert.brown@itproject.ca</t>
+  </si>
+  <si>
+    <t>david.jones@itproject.ca</t>
+  </si>
+  <si>
+    <t>william.garcia@itproject.ca</t>
+  </si>
+  <si>
+    <t>mary.miller@itproject.ca</t>
+  </si>
+  <si>
+    <t>maria.davis@itproject.ca</t>
+  </si>
+  <si>
+    <t>joseph.martinez@itproject.ca</t>
+  </si>
+  <si>
+    <t>maya.bennett@itproject.ca</t>
+  </si>
+  <si>
+    <t>ava.collins@itproject.ca</t>
+  </si>
+  <si>
+    <t>layla.cooper@itproject.ca</t>
+  </si>
+  <si>
+    <t>owen.blake@itproject.ca</t>
+  </si>
+  <si>
+    <t>jane.doe@itproject.ca</t>
+  </si>
+  <si>
+    <t>noah.parker@itproject.ca</t>
+  </si>
+  <si>
+    <t>ethan.brooks@itproject.ca</t>
+  </si>
+  <si>
+    <t>mason.wright@itproject.ca</t>
+  </si>
+  <si>
+    <t>aria.sullivan@itproject.ca</t>
+  </si>
+  <si>
+    <t>chloe.reed@itproject.ca</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Accounting</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Supply Chain</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Legal</t>
+  </si>
+  <si>
+    <t>Remote</t>
+  </si>
+  <si>
+    <t>Hybrid</t>
+  </si>
+  <si>
+    <t>Desktop</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>Alex Zimmer</t>
+  </si>
+  <si>
+    <t>alex.zimmer@itproject.ca</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy A54</t>
+  </si>
+  <si>
+    <t>R9JK20M4LPQ</t>
+  </si>
+  <si>
+    <t>iPhone 14</t>
+  </si>
+  <si>
+    <t>F7MP8Y2WRT</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy S22</t>
+  </si>
+  <si>
+    <t>R58N40K2PQR</t>
+  </si>
+  <si>
+    <t>iPhone 13</t>
+  </si>
+  <si>
+    <t>F2LN3X9JQP</t>
+  </si>
+  <si>
+    <t>Dell KB216 Keyboard</t>
+  </si>
+  <si>
+    <t>DL4492MK7</t>
+  </si>
+  <si>
+    <t>Logitech MK540 Combo</t>
+  </si>
+  <si>
+    <t>2217LZ093841</t>
+  </si>
+  <si>
+    <t>Microsoft Sculpt Keyboard</t>
+  </si>
+  <si>
+    <t>MS7K2019X4</t>
+  </si>
+  <si>
+    <t>Logitech MX Master 3S</t>
+  </si>
+  <si>
+    <t>2318LZ048392</t>
+  </si>
+  <si>
+    <t>Samsung S24R350</t>
+  </si>
+  <si>
+    <t>HL9K203M7</t>
+  </si>
+  <si>
+    <t>LG 27UL850-W</t>
+  </si>
+  <si>
+    <t>802NTDK4Y123</t>
+  </si>
+  <si>
+    <t>HP E24 G5</t>
+  </si>
+  <si>
+    <t>6CM1023PQR</t>
+  </si>
+  <si>
+    <t>Dell P2422H</t>
+  </si>
+  <si>
+    <t>CN-0K8M2P-74261</t>
+  </si>
+  <si>
+    <t>Dell OptiPlex 5090</t>
+  </si>
+  <si>
+    <t>Lenovo ThinkCentre M90t</t>
+  </si>
+  <si>
+    <t>HP ProDesk 600 G9</t>
+  </si>
+  <si>
+    <t>Dell OptiPlex 7010</t>
+  </si>
+  <si>
+    <t>3H8N2YV7</t>
+  </si>
+  <si>
+    <t>8CJ4452LMN</t>
+  </si>
+  <si>
+    <t>MP2K8XR4</t>
+  </si>
+  <si>
+    <t>6T9D3QZ2</t>
+  </si>
+  <si>
+    <t>Unused</t>
+  </si>
+  <si>
+    <t>Faulty</t>
+  </si>
+  <si>
+    <t>Retired</t>
+  </si>
+  <si>
+    <t>Returned device</t>
+  </si>
+  <si>
+    <t>Spare device</t>
+  </si>
+  <si>
+    <t>Awaiting for new hire</t>
+  </si>
+  <si>
+    <t>Dead battery</t>
+  </si>
+  <si>
+    <t>Device outdated</t>
+  </si>
+  <si>
+    <t>Employee left company</t>
+  </si>
+  <si>
+    <t>Dead pixels on monitor screen</t>
+  </si>
+  <si>
+    <t>Cracked screen on device</t>
+  </si>
+  <si>
     <t>LT-0001</t>
   </si>
   <si>
@@ -90,172 +405,52 @@
     <t>LT-0004</t>
   </si>
   <si>
-    <t>7K2L9X3</t>
-  </si>
-  <si>
-    <t>5CD2371XYZ</t>
-  </si>
-  <si>
-    <t>PF3K9RT2</t>
-  </si>
-  <si>
-    <t>9M4P2WQ1</t>
-  </si>
-  <si>
-    <t>HP EliteBook 840 G9</t>
-  </si>
-  <si>
-    <t>Lenovo ThinkPad T14</t>
-  </si>
-  <si>
-    <t>Dell Latitude 7420</t>
-  </si>
-  <si>
-    <t>James Johnson</t>
-  </si>
-  <si>
-    <t>John Williams</t>
-  </si>
-  <si>
-    <t>Robert Brown</t>
-  </si>
-  <si>
-    <t>David Jones</t>
-  </si>
-  <si>
-    <t>William Garcia</t>
-  </si>
-  <si>
-    <t>Mary Miller</t>
-  </si>
-  <si>
-    <t>Maria Davis</t>
-  </si>
-  <si>
-    <t>Joseph Martinez</t>
-  </si>
-  <si>
-    <t>Bilal Akhtar</t>
-  </si>
-  <si>
-    <t>Maya Bennett</t>
-  </si>
-  <si>
-    <t>Ava Collins</t>
-  </si>
-  <si>
-    <t>Layla Cooper</t>
-  </si>
-  <si>
-    <t>Owen Blake</t>
-  </si>
-  <si>
-    <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>Noah Parker</t>
-  </si>
-  <si>
-    <t>Ethan Brooks</t>
-  </si>
-  <si>
-    <t>Mason Wright</t>
-  </si>
-  <si>
-    <t>Aria Sullivan</t>
-  </si>
-  <si>
-    <t>Chloe Reed</t>
-  </si>
-  <si>
-    <t>bilal.akhtar@itproject.ca</t>
-  </si>
-  <si>
-    <t>james.johnson@itproject.ca</t>
-  </si>
-  <si>
-    <t>john.williams@itproject.ca</t>
-  </si>
-  <si>
-    <t>robert.brown@itproject.ca</t>
-  </si>
-  <si>
-    <t>david.jones@itproject.ca</t>
-  </si>
-  <si>
-    <t>william.garcia@itproject.ca</t>
-  </si>
-  <si>
-    <t>mary.miller@itproject.ca</t>
-  </si>
-  <si>
-    <t>maria.davis@itproject.ca</t>
-  </si>
-  <si>
-    <t>joseph.martinez@itproject.ca</t>
-  </si>
-  <si>
-    <t>maya.bennett@itproject.ca</t>
-  </si>
-  <si>
-    <t>ava.collins@itproject.ca</t>
-  </si>
-  <si>
-    <t>layla.cooper@itproject.ca</t>
-  </si>
-  <si>
-    <t>owen.blake@itproject.ca</t>
-  </si>
-  <si>
-    <t>jane.doe@itproject.ca</t>
-  </si>
-  <si>
-    <t>noah.parker@itproject.ca</t>
-  </si>
-  <si>
-    <t>ethan.brooks@itproject.ca</t>
-  </si>
-  <si>
-    <t>mason.wright@itproject.ca</t>
-  </si>
-  <si>
-    <t>aria.sullivan@itproject.ca</t>
-  </si>
-  <si>
-    <t>chloe.reed@itproject.ca</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>Finance</t>
-  </si>
-  <si>
-    <t>Accounting</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>Supply Chain</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Legal</t>
-  </si>
-  <si>
-    <t>Remote</t>
-  </si>
-  <si>
-    <t>Hybrid</t>
+    <t>DT-0001</t>
+  </si>
+  <si>
+    <t>DT-0002</t>
+  </si>
+  <si>
+    <t>DT-0003</t>
+  </si>
+  <si>
+    <t>DT-0004</t>
+  </si>
+  <si>
+    <t>MN-0001</t>
+  </si>
+  <si>
+    <t>MN-0002</t>
+  </si>
+  <si>
+    <t>MN-0003</t>
+  </si>
+  <si>
+    <t>PR-0004</t>
+  </si>
+  <si>
+    <t>MN-0004</t>
+  </si>
+  <si>
+    <t>PR-0001</t>
+  </si>
+  <si>
+    <t>PR-0002</t>
+  </si>
+  <si>
+    <t>PR-0003</t>
+  </si>
+  <si>
+    <t>MB-0001</t>
+  </si>
+  <si>
+    <t>MB-0002</t>
+  </si>
+  <si>
+    <t>MB-0003</t>
+  </si>
+  <si>
+    <t>MB-0004</t>
   </si>
 </sst>
 </file>
@@ -360,7 +555,24 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -638,13 +850,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="27.7109375" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
@@ -694,7 +906,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>122</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>12</v>
@@ -703,13 +915,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -718,10 +930,10 @@
         <v>15</v>
       </c>
       <c r="I2" s="4">
-        <v>45306</v>
+        <v>43907</v>
       </c>
       <c r="J2" s="4">
-        <v>46402</v>
+        <v>45002</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>16</v>
@@ -730,414 +942,650 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I3" s="4">
-        <v>44973</v>
-      </c>
-      <c r="J3" s="4"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
+        <v>44413</v>
+      </c>
+      <c r="J3" s="4">
+        <v>45509</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="I4" s="4">
+        <v>44888</v>
+      </c>
+      <c r="J4" s="4">
+        <v>45984</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>125</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="2"/>
+      <c r="I5" s="4">
+        <v>44971</v>
+      </c>
+      <c r="J5" s="4">
+        <v>46067</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="E6" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="I6" s="4">
+        <v>44011</v>
+      </c>
+      <c r="J6" s="4">
+        <v>45106</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="2"/>
+      <c r="I7" s="4">
+        <v>45546</v>
+      </c>
+      <c r="J7" s="4">
+        <v>46641</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="E8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="4">
+        <v>44203</v>
+      </c>
+      <c r="J8" s="4">
+        <v>45298</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="4">
+        <v>44913</v>
+      </c>
+      <c r="J9" s="4">
+        <v>46009</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="4">
+        <v>45773</v>
+      </c>
+      <c r="J10" s="4">
+        <v>46869</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F11" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
+      <c r="I11" s="4">
+        <v>44015</v>
+      </c>
+      <c r="J11" s="4">
+        <v>45110</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>98</v>
+      </c>
       <c r="E12" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="I12" s="4">
+        <v>44484</v>
+      </c>
+      <c r="J12" s="4">
+        <v>45580</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="E13" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="2"/>
+      <c r="I13" s="4">
+        <v>45067</v>
+      </c>
+      <c r="J13" s="4">
+        <v>46163</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L13" s="2"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="E14" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="2"/>
+      <c r="I14" s="4">
+        <v>44601</v>
+      </c>
+      <c r="J14" s="4">
+        <v>45697</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L14" s="2"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="E15" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="2"/>
+      <c r="I15" s="4">
+        <v>45531</v>
+      </c>
+      <c r="J15" s="4">
+        <v>46626</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L15" s="2"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E16" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="I16" s="4">
+        <v>44141</v>
+      </c>
+      <c r="J16" s="4">
+        <v>45236</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="E17" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="I17" s="4">
+        <v>45746</v>
+      </c>
+      <c r="J17" s="4">
+        <v>46842</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L17" s="2"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E18" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
+        <v>71</v>
+      </c>
+      <c r="I18" s="4">
+        <v>44359</v>
+      </c>
+      <c r="J18" s="4">
+        <v>45455</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="E19" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="I19" s="4">
+        <v>44828</v>
+      </c>
+      <c r="J19" s="4">
+        <v>45924</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L19" s="2"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="A20" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="E20" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
@@ -1145,25 +1593,77 @@
       <c r="H20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="2"/>
+      <c r="I20" s="4">
+        <v>45310</v>
+      </c>
+      <c r="J20" s="4">
+        <v>46406</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="L20" s="2"/>
     </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="4">
+        <v>43929</v>
+      </c>
+      <c r="J21" s="4">
+        <v>45024</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="K2 X3 W4:W20">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Retired">
+  <conditionalFormatting sqref="K2:K21">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Retired">
       <formula>NOT(ISERROR(SEARCH("Retired",K2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Faulty">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Faulty">
       <formula>NOT(ISERROR(SEARCH("Faulty",K2)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="X3 W4:W20">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Retired">
+      <formula>NOT(ISERROR(SEARCH("Retired",W3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Faulty">
+      <formula>NOT(ISERROR(SEARCH("Faulty",W3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B20" xr:uid="{65971D14-0A3A-42EF-AE89-968C8A23BBDA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B21" xr:uid="{65971D14-0A3A-42EF-AE89-968C8A23BBDA}">
       <formula1>"Laptop, Desktop, Monitor, Peripheral, Mobile"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K20" xr:uid="{D395B214-B837-45E2-AD8D-5AAA424B774B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K21" xr:uid="{D395B214-B837-45E2-AD8D-5AAA424B774B}">
       <formula1>"In Use, Unused, Faulty, Retired"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1187,6 +1687,7 @@
     <hyperlink ref="F18" r:id="rId17" xr:uid="{872412FB-CA74-4606-8D6A-45E35C56FD17}"/>
     <hyperlink ref="F19" r:id="rId18" xr:uid="{A5D050D6-FA8E-4B6B-A7B6-B5C4E622FAE5}"/>
     <hyperlink ref="F20" r:id="rId19" xr:uid="{A4E2B197-A800-4FA6-9DAA-C86208289327}"/>
+    <hyperlink ref="F21" r:id="rId20" xr:uid="{A8F37923-FB9E-4634-A682-4B42E2A18E2B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>